<commit_message>
🔪 Slice france_travail 2026-09-16
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,32 +714,32 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Durée de 980 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -749,17 +749,17 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>http://www.insup.org/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>prf@insup.org</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>prf@insup.org | paysmontois@insup.org | nrousseau@insup.org</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -774,48 +774,40 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>0558068971</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>0558068971</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis - 4 hModule 3 CCP 1 Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Veille professionnelle et commerciale : L'Entreprise et son environnement, Droit commercial, Stratégies commerciales, E-commerce et digitalisation du point de vente, Usages professionnels dans le respect du Développement durable et de la Politique RSE, Spécialisation Univers produit Gestion des flux : Logistique du point de vente, Réception des marchandises, Gestes et postures Contribuer au merchandising : Promotions et animation commerciale, Introduction au merchandising d'organisation et séductionAnalyse des performances commerciales : Tableaux de bord, Règles d'implantations - 315 hModule 4 CCP 2 : Améliorer l'expérience client dans un environnement omnicanal - Valorisation de l'image de l'unité marchande : Communication et image de marque, Réseaux sociaux et professionnels, E-réputation, Outils et applicatifs numériques - Vente connectée, Commandes en ligneConduite d'entretien de vente (produits/services) : Connaissance de la clientèle, Posture de service, Techniques d'entretien, Gestion du Click § CollectSuivi des ventes : Indicateurs commerciaux, Tableau de bord , Analyse commerciale, Plan d'actionFidélisation et consolidation de l'expérience client : Enjeux et techniques de fidél | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
-        </is>
-      </c>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr"/>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913194/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,32 +819,32 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>40100 Dax</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>3 Rue DES SALINES | 40100 Dax | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Durée de 805 heures (dont 315 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -862,17 +854,17 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>http://www.insup.org/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>prf@insup.org</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>prf@insup.org | paysdacquois@insup.org</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -887,48 +879,40 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>0558917868</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>0558917868</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr"/>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis - 4 hModule 3 CCP 1 Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Veille professionnelle et commerciale : L'Entreprise et son environnement, Droit commercial, Stratégies commerciales, E-commerce et digitalisation du point de vente, Usages professionnels dans le respect du Développement durable et de la Politique RSE, Spécialisation Univers produit Gestion des flux : Logistique du point de vente, Réception des marchandises, Gestes et postures Contribuer au merchandising : Promotions et animation commerciale, Introduction au merchandising d'organisation et séductionAnalyse des performances commerciales : Tableaux de bord, Règles d'implantations - 315 hModule 4 CCP 2 : Améliorer l'expérience client dans un environnement omnicanal - Valorisation de l'image de l'unité marchande : Communication et image de marque, Réseaux sociaux et professionnels, E-réputation, Outils et applicatifs numériques - Vente connectée, Commandes en ligneConduite d'entretien de vente (produits/services) : Connaissance de la clientèle, Posture de service, Techniques d'entretien, Gestion du Click § CollectSuivi des ventes : Indicateurs commerciaux, Tableau de bord , Analyse commerciale, Plan d'actionFidélisation et consolidation de l'expérience client : Enjeux et techniques de fidél | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913202/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -940,32 +924,32 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Employé(e)commercial (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE | 362 Boulevard du chemin creux | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 770 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -975,17 +959,17 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>http://www.insup.org/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>prf@insup.org</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>prf@insup.org | centre.tertiaire.montdemarsan@greta-cfa-aquitaine.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1000,12 +984,12 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0558056569</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0558056569</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
@@ -1015,33 +999,33 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Approvisionnement de l'unité marchande : L'entreprise, Règlementation, Stratégies commerciales, Usages professionnels conformes au développement durable et à la politique RSE, Logistique, Hygiène/sécurité alimentaire, Réception et préparation des marchandises, ManutentionPrésentation marchande des produits : Univers produits, Merchandising d'organisation et séduction Contribution à la gestion et optimisation des stocks : Suivi des stocks, Démarque/surmarque, Inventaires, E-Commerce et digitalisation (NAVA)Traitement des commandes : Gestion des commandes faites en ligne ou sur place - 196 hModule 4 CCP 2 : Accueillir les clients et répondre à leur demande dans un environnement omnicanal - Accueil et service clients : Typologie clientèle, Techniques de communication, Informer, orienter et conseiller, Gestion des retraits des commandes internet et Drive, FidélisationContribution à l'amélioration de l'expérience d'achat :Prendre en charge et accompagner les clients (aide au parcours d'achat)Tenue d'un poste de caisse et supervision des caisses libre-service : Utilisation des matériels (caisse, balance, TPE... Rè | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913205/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1053,32 +1037,32 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de reconditionnement numérique (TP) [HSP 1er NQ]</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1088,17 +1072,17 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>contact@afec.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | formation-mont_de_marsan@afpa.fr</t>
+          <t>cergy@afec.fr | contact@afec.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1113,48 +1097,40 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0143388885</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0143388885</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>TP IDI-Période d'intégration - Intégrer son groupe et sa formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelRepérer les risques liés à l'exercice du métier et se sensibiliser au développement durableDévelopper son efficacité personnelleS'inscrire dans une perspective d'emploi - 35 hTP IDI-Connaissances communes IDI - Utilisation Informatique - Internet et bureautiqueAnglais TechniquePosture ProfessionnelleSensibilisation aux règles : Electriques, DEEE, RGPD - 140 hTP IDI-Mettre en service des équipements informatiques fixes et mobiles - Installer un système ou déployer une image sur un poste client fixe ou mobileConfigurer, paramétrer et personnaliser un équipement informatique fixe ou mobileRaccorder un équipement fixe ou mobile à un réseauInformer et conseiller le client ou l'utilisateur - 245 hTP IDI-Dépanner et reconditionner des équipements informatiques fixes et mobiles - Diagnostiquer et résoudre un dysfonctionnement d'un équipement informatique fixe ou mobileVérifier, identifier, trier un équipement informatique fixe ou mobile d'occasionRevaloriser et intégrer un équipement fixe ou mobile - 175 hTP IDI-Période d'application en entreprise IDI - Période entreprise IDI - 140 hTP IDI-Période Certification IDI - Séquence de certification IDI - 35 hTP IDI-Sensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP IDI-Sensibilisation aux enjeux des valeurs de la république - APPRÉHENDERRecontextualisation du principe de laïcité. Présentation : liberté, égalité, fraternité, laïcité, etcAGIRCulture du discernement et de la nuance, acceptation des différences. Prendre conscience de ses responsabilités. Agir individuellement au quotidien dans les valeurs de la République et de la citoyennetéComprendre la discrimination et ses différentes formes (fe | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de reconditionnement numérique</t>
-        </is>
-      </c>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr"/>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10919990/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1166,32 +1142,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Assistant(e) de vie dépendance et handicap [HSP 1er NQ]</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE | 36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1201,17 +1177,17 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | paysmontois@insup.org | nrousseau@insup.org</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1226,48 +1202,40 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>0558068971</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>0558068971</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>ACCUEIL ET INTEGRATION DANS LA FORMATION - "Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables" - 70 h"DÉVELOPPEMENT DE SON ACTIVITÉ PROFESSIONNELLE AUPRÈS DE PLUSIEURS PARTICULIERS EMPLOYEURS" - "S'initier à l'informatique et à InternetEtre autonome dans sa recherche d'emploi en intégrant les outils numériquesDévelopper son réseau et réaliser une veille sur son secteur d'activité - 49 h"GESTION DE SON ACTIVITÉ PROFESSIONNELLE AUPRÈS DE PARTICULIERS EMPLOYEURS " - "Droits et devoirs dans l'exercice de son métierLes clés d'un entretien réussi avec un particulier employeurLes clés d'une bonne relation de travail avec le particulier employeur : communication et organisation - 49 hPRÉVENTION ET SÉCURITÉ AU DOMICILE - "Organisation, aménagement et sécurisation de l'espace professionnelPrévenir les risques professionnels et sécuriser son intervention - 42 hENTRETIEN DU DOMICILE ET DU LINGE : PRATIQUES ÉCORESPONSABLES - "Entretien du cadre de vie et pratiques écoresponsablesEntretien du linge et pratiques écoresponsables " - 42 h"PERSONNE AGÉE EN SITUATION DE DÉPENDANCE : ACCOMPAGNEMENT PERSONNALISÉ " - "Les droits de la personne âgée dépendante et les fondements d'une démarche de bientraitanceComprendre les pathologies liées au vieillissement pour un accompagnement de qualité S'inscrire dans une démarche de projet personnalisé et travailler en collaboration pour mieux accompagner la personne en situation de dépendance - 56 h"PERSONNE EN SITUATION DE HANDICAP : PROJET ET ACCOMPAGNEMENT PERSONNALISÉ" - "Les droits de la personne en situation de handicap et les fondements d'une démarche de bientraitance Comprendre le handicap pour mieux accompagner la personne S'inscrire dans une démarche de projet personnalisé et travailler en collaboration pour mieux accompagner la personne en situation de dépendance - 56 hACTES DU QUOTIDIEN ET ACTIVITÉS DE L'ADULTE EN SITUATION DE DÉPENDANCE - "Accompagner une personne en situation de dépendance dans les actes d'hygiène et de confortTransferts et déplacements d'une personne en situation de dépendance Accompagner une personne en situation de dépendance dans ses loisirs" - 56 | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Assistant de vie dépendance et handicap</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10925810/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1279,32 +1247,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE | 36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1314,17 +1282,17 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | paysmontois@insup.org | nrousseau@insup.org</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1339,48 +1307,40 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0558068971</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0558068971</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre équipe, Visite du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification visée, Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action. - 17 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Réaliser une prestation de nettoyage manuel - Environnement professionnel : le nettoyage industriel Prévention des risques : Règles d'hygiène et de sécurité, EPI, Gestuelle métier, Dysfonctionnements et risques associésNettoyage manuel : Techniques de nettoyage, Choix et utilisation des produits, Lavage des surfaces vitrées, Dépoussiérage des surfaces et sols, Nettoyage, Désinfection, Détartrage des sanitaires, Protocoles de bionettoyage en environnement spécifique Respect des standards de qualité : Contrôle de sa prestationIntégration des principes du développement durablePosture professionnelle adaptée - 245 hModule 4 CCP 2 Réaliser une prestation de nettoyage ou de remise en état mécanisée - Prévention des risques : Hygiène et Sécurité, Gestuelle, DysfonctionnementsRevêtements de sols : caractéristiquesProduits écologiques / écogestesUtilisation du matériel professionnel : Autolaveuse et monobrosseTechniques de nettoyage ou de remise en état mécanisé : Lavages mécanisés, méthode spray, lustrage et spray moquette - Remise en état - Récurage - Décapage - Métallisation - Shampoin | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10925813/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1392,32 +1352,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>40100 Dax</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>INSUP AQUITAINE | 3 Rue DES SALINES | 40100 Dax | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1427,17 +1387,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | paysdacquois@insup.org | landes@insup.org</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1452,48 +1412,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0558917868</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0558917868</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre équipe, Visite du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification visée, Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action. - 17 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Réaliser une prestation de nettoyage manuel - Environnement professionnel : le nettoyage industriel Prévention des risques : Règles d'hygiène et de sécurité, EPI, Gestuelle métier, Dysfonctionnements et risques associésNettoyage manuel : Techniques de nettoyage, Choix et utilisation des produits, Lavage des surfaces vitrées, Dépoussiérage des surfaces et sols, Nettoyage, Désinfection, Détartrage des sanitaires, Protocoles de bionettoyage en environnement spécifique Respect des standards de qualité : Contrôle de sa prestationIntégration des principes du développement durablePosture professionnelle adaptée - 245 hModule 4 CCP 2 Réaliser une prestation de nettoyage ou de remise en état mécanisée - Prévention des risques : Hygiène et Sécurité, Gestuelle, DysfonctionnementsRevêtements de sols : caractéristiquesProduits écologiques / écogestesUtilisation du matériel professionnel : Autolaveuse et monobrosseTechniques de nettoyage ou de remise en état mécanisé : Lavages mécanisés, méthode spray, lustrage et spray moquette - Remise en état - Récurage - Décapage - Métallisation - Shampoin | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10925829/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1505,32 +1457,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de maintenance des bâtiments (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1540,17 +1492,17 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1565,12 +1517,12 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -1580,33 +1532,33 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>TP AMB Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP AMB Bloc de compétences : Assurer la maintenance courante des aménagements intérieurs d'un bâtiment - Effectuer la maintenance améliorative courante des aménagements intérieurs d'un bâtiment Effectuer la maintenance améliorative courante des revêtements intérieurs d'un bâtiment Effectuer la maintenance préventive courante des menuiseries et fermetures d'un bâtiment Effectuer la maintenance corrective courante des aménagements intérieurs d'un bâtiment - 280 hTP AMB Période 1 en entreprise - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 70 hTP AMB Bloc de compétences : Assurer la maintenance courante de l'installation et des équipements électriques d'un bâtiment - Effectuer la maintenance améliorative courante d'une installation électrique monophasée d'un bâtiment Effectuer la maintenance préventive courante de l'installation et des équipements électriques d'un bâtiment Effectuer la maintenance corrective courante de l'installation et des équipements électriques d'un bâtiment - 175 hTP AMB Bloc de compétences : Assurer la maintenance courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment - Effectuer la maintenance améliorative courante de l'installation sanitaire d'un bâtiment Effectuer la maintenance préventive courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment Effectuer la maintenance corrective courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment - 140 hTP AMB Période 2 en entreprise - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP AMB Période de certification - Epreuve de certification - 35 hTP AMB Sensibi | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de maintenance des bâtiments</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10928110/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1618,32 +1570,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Action Préparatoire aux métiers du BTP [HSP 1er NQ]</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1653,17 +1605,17 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1678,40 +1630,48 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0619257169</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr"/>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Période d'intégration - Intégrer son groupe et sa formationS'approprier le cadre et les objectifs de la formation préparatoire Développer sa culture numérique et prendre en main la plateforme MètisDécouvrir la boîte à outils numériqueDécouvrir Mètis et se repérer dans son parcoursPasser les tests de positionnementPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une continuité de parcours certifiant ou une perspective d'emploi, un contrat en alternanceInitier son portefeuille de compétences - 35 hModule 1 : Découverte des métiers du secteur BTP et de leurs évolutions - Immersions sur les plateaux de formation - Découverte des métiers Les travaux publics : Canalisateur, maçon voirie réseaux divers, conducteur d'engins... Le gros oeuvre : Maçon, charpentier, couvreur zingueur... Le second oeuvre : Peintre, Carreleur, agent de maintenance des bâtiments, plombier, électricien, menuisier...Visites d'entreprises : Préparer, réaliser et exploiter une visite en entreprise Participation à des évènementiels Salons, jobs dating à partir d'une préparation collectiveMatinale entreprise (témoignages professionnels)BILAN INDIVIDUEL D'ORIENTATION - 70 hModule 2 : Acquérir le socle des connaissances nécessaires pour aller vers les métiers de l'industrie - Se remettre à niveau en mathématiquesUtiliser le système métriqueApprendre à lire des documents techniques, des plans....Développer sa communication écrite, son expression orale, comprendre les règles et instructionsTravailler en équipe et adopter la posture professionnelle attendueBILAN INDIVIDUEL D'ORIENTATION - 70 hModule 3 : Acquérir les bases des connaissances techniques et les gestes professionnels d'un métier - Réaliser un ouvrage simple en tenant compte des exigences de sécurité Identifier le matériel et les équipements nécessaires à la réalisation d'un ouvrage simplePréparer la matière nécessaire à la réalisation d'un ouvrage simpleRéaliser un ouvrage simpleMaintenir, l'organisation et la propreté du poste de travailTravailler en sécurité et conformément à la réglementation Repérer les risques liés à l'exercice des métiers de l'industrie Se sensibiliser au développement durable dans les métiers du BTPBILAN INDIVIDUEL D'ORIENTATION - 105 hModule 4 : Acco | Organisme | DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE | http://www.afpa.fr | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr"/>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+        </is>
+      </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10928111/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1723,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Monteur, monteuse en installation thermique et sanitaire (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>40000 Mont-de-Marsan</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1758,17 +1718,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>contact@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
+          <t>cergy@afec.fr | contact@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1783,12 +1743,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0143388885</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0619257169</t>
+          <t>0143388885</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1798,33 +1758,33 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>TP ITS Période d'intégration - Intégrer son groupe et sa formationS'inscrire dans une perspective d'emploiPréciser ses besoins de formation et contractualiser son parcours personnaliséDévelopper son autonomie en formationS'approprier les objectifs de la formation et repérer son futur environnement professionnel - 35 hTP ITS Bloc de compétences : Réaliser des installations sanitaire de bâtiments - Installer des équipements de renouvellement d'air dans des locaux d'habitation Effectuer l'analyse et établir le mode opératoireInstaller un système d'extraction dans des bâtiments à usage d'habitation individuelle et collectifsInstaller des appareils sanitaires Effectuer l' analyse de la mise en oeuvre de travaux d'installation d'appareil sanitaireInstaller des équipements de production d'eau chaude sanitaireRéaliser l'installation d'un équipement de production ECS solaire individuel et collectif, à gaz - 350 hTP ITS Période en entreprise-1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 70 hTP ITS Bloc de Compétences : Réaliser des installations de chauffage dans des locaux d'habitation - Installer des émetteurs de chaleur en tube cuivre et matériaux de synthèse Effectuer l' analyse de la mise en oeuvre de travaux de chauffageRéaliser l'installation d' un plancher chauffant basse température Modifier un réseau de chauffage existant Établir un mode opératoire pour intervenir sur une installation de chauffage existanteInstaller un générateur de chauffage dans des locaux d'habitation - 350 hTP ITS Période en entreprise-2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 105 hTP ITS Période de Certification - Certification - 35 hTP ITS Sensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'a | Validation | Type de validation : | Diplôme autres ministères | Certifications :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certifications : | Titre professionnel plombier chauffagiste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10928127/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1836,32 +1796,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>INSUP AQUITAINE</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 980 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1871,17 +1831,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.insup.org/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>prf@insup.org</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>prf@insup.org | paysmontois@insup.org | nrousseau@insup.org</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1896,40 +1856,48 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0558068971</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr"/>
+          <t>0558068971</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr"/>
+          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis - 4 hModule 3 CCP 1 Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Veille professionnelle et commerciale : L'Entreprise et son environnement, Droit commercial, Stratégies commerciales, E-commerce et digitalisation du point de vente, Usages professionnels dans le respect du Développement durable et de la Politique RSE, Spécialisation Univers produit Gestion des flux : Logistique du point de vente, Réception des marchandises, Gestes et postures Contribuer au merchandising : Promotions et animation commerciale, Introduction au merchandising d'organisation et séductionAnalyse des performances commerciales : Tableaux de bord, Règles d'implantations - 315 hModule 4 CCP 2 : Améliorer l'expérience client dans un environnement omnicanal - Valorisation de l'image de l'unité marchande : Communication et image de marque, Réseaux sociaux et professionnels, E-réputation, Outils et applicatifs numériques - Vente connectée, Commandes en ligneConduite d'entretien de vente (produits/services) : Connaissance de la clientèle, Posture de service, Techniques d'entretien, Gestion du Click § CollectSuivi des ventes : Indicateurs commerciaux, Tableau de bord , Analyse commerciale, Plan d'actionFidélisation et consolidation de l'expérience client : Enjeux et techniques de fidél | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+        </is>
+      </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913194/true/false/false/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1941,32 +1909,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>INSUP AQUITAINE</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40100 Dax</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>3 Rue DES SALINES | 40100 Dax | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 805 heures (dont 315 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1976,17 +1944,17 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.insup.org/</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>prf@insup.org</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>prf@insup.org | paysdacquois@insup.org</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -2001,40 +1969,48 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0558917868</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr"/>
+          <t>0558917868</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr"/>
+          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis - 4 hModule 3 CCP 1 Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Veille professionnelle et commerciale : L'Entreprise et son environnement, Droit commercial, Stratégies commerciales, E-commerce et digitalisation du point de vente, Usages professionnels dans le respect du Développement durable et de la Politique RSE, Spécialisation Univers produit Gestion des flux : Logistique du point de vente, Réception des marchandises, Gestes et postures Contribuer au merchandising : Promotions et animation commerciale, Introduction au merchandising d'organisation et séductionAnalyse des performances commerciales : Tableaux de bord, Règles d'implantations - 315 hModule 4 CCP 2 : Améliorer l'expérience client dans un environnement omnicanal - Valorisation de l'image de l'unité marchande : Communication et image de marque, Réseaux sociaux et professionnels, E-réputation, Outils et applicatifs numériques - Vente connectée, Commandes en ligneConduite d'entretien de vente (produits/services) : Connaissance de la clientèle, Posture de service, Techniques d'entretien, Gestion du Click § CollectSuivi des ventes : Indicateurs commerciaux, Tableau de bord , Analyse commerciale, Plan d'actionFidélisation et consolidation de l'expérience client : Enjeux et techniques de fidél | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+        </is>
+      </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913202/true/false/false/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2046,32 +2022,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Employé(e)commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>INSUP AQUITAINE</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>GRETA CFA AQUITAINE | 362 Boulevard du chemin creux | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 770 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2081,17 +2057,17 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.insup.org/</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>prf@insup.org</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>prf@insup.org | centre.tertiaire.montdemarsan@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2106,12 +2082,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0558056569</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0558056569</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2121,33 +2097,33 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre de l'équipe, Découverte du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification , Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action - 18 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Approvisionnement de l'unité marchande : L'entreprise, Règlementation, Stratégies commerciales, Usages professionnels conformes au développement durable et à la politique RSE, Logistique, Hygiène/sécurité alimentaire, Réception et préparation des marchandises, ManutentionPrésentation marchande des produits : Univers produits, Merchandising d'organisation et séduction Contribution à la gestion et optimisation des stocks : Suivi des stocks, Démarque/surmarque, Inventaires, E-Commerce et digitalisation (NAVA)Traitement des commandes : Gestion des commandes faites en ligne ou sur place - 196 hModule 4 CCP 2 : Accueillir les clients et répondre à leur demande dans un environnement omnicanal - Accueil et service clients : Typologie clientèle, Techniques de communication, Informer, orienter et conseiller, Gestion des retraits des commandes internet et Drive, FidélisationContribution à l'amélioration de l'expérience d'achat :Prendre en charge et accompagner les clients (aide au parcours d'achat)Tenue d'un poste de caisse et supervision des caisses libre-service : Utilisation des matériels (caisse, balance, TPE... Rè | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913205/true/false/false/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2159,32 +2135,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>Agent(e) de reconditionnement numérique (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>AFEC</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2194,17 +2170,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>cergy@afec.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>cergy@afec.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | formation-mont_de_marsan@afpa.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2219,40 +2195,48 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0143388881</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0143388881</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="inlineStr"/>
+          <t>0619257169</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T15" s="7" t="inlineStr"/>
+          <t>TP IDI-Période d'intégration - Intégrer son groupe et sa formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelRepérer les risques liés à l'exercice du métier et se sensibiliser au développement durableDévelopper son efficacité personnelleS'inscrire dans une perspective d'emploi - 35 hTP IDI-Connaissances communes IDI - Utilisation Informatique - Internet et bureautiqueAnglais TechniquePosture ProfessionnelleSensibilisation aux règles : Electriques, DEEE, RGPD - 140 hTP IDI-Mettre en service des équipements informatiques fixes et mobiles - Installer un système ou déployer une image sur un poste client fixe ou mobileConfigurer, paramétrer et personnaliser un équipement informatique fixe ou mobileRaccorder un équipement fixe ou mobile à un réseauInformer et conseiller le client ou l'utilisateur - 245 hTP IDI-Dépanner et reconditionner des équipements informatiques fixes et mobiles - Diagnostiquer et résoudre un dysfonctionnement d'un équipement informatique fixe ou mobileVérifier, identifier, trier un équipement informatique fixe ou mobile d'occasionRevaloriser et intégrer un équipement fixe ou mobile - 175 hTP IDI-Période d'application en entreprise IDI - Période entreprise IDI - 140 hTP IDI-Période Certification IDI - Séquence de certification IDI - 35 hTP IDI-Sensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP IDI-Sensibilisation aux enjeux des valeurs de la république - APPRÉHENDERRecontextualisation du principe de laïcité. Présentation : liberté, égalité, fraternité, laïcité, etcAGIRCulture du discernement et de la nuance, acceptation des différences. Prendre conscience de ses responsabilités. Agir individuellement au quotidien dans les valeurs de la République et de la citoyennetéComprendre la discrimination et ses différentes formes (fe | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de reconditionnement numérique</t>
+        </is>
+      </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10919990/true/false/false/true</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2264,32 +2248,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Assistant(e) de vie dépendance et handicap [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>INSUP AQUITAINE | 36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2299,17 +2283,17 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | paysmontois@insup.org | nrousseau@insup.org</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2324,40 +2308,48 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0558068971</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr"/>
+          <t>0558068971</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr"/>
+          <t>ACCUEIL ET INTEGRATION DANS LA FORMATION - "Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables" - 70 h"DÉVELOPPEMENT DE SON ACTIVITÉ PROFESSIONNELLE AUPRÈS DE PLUSIEURS PARTICULIERS EMPLOYEURS" - "S'initier à l'informatique et à InternetEtre autonome dans sa recherche d'emploi en intégrant les outils numériquesDévelopper son réseau et réaliser une veille sur son secteur d'activité - 49 h"GESTION DE SON ACTIVITÉ PROFESSIONNELLE AUPRÈS DE PARTICULIERS EMPLOYEURS " - "Droits et devoirs dans l'exercice de son métierLes clés d'un entretien réussi avec un particulier employeurLes clés d'une bonne relation de travail avec le particulier employeur : communication et organisation - 49 hPRÉVENTION ET SÉCURITÉ AU DOMICILE - "Organisation, aménagement et sécurisation de l'espace professionnelPrévenir les risques professionnels et sécuriser son intervention - 42 hENTRETIEN DU DOMICILE ET DU LINGE : PRATIQUES ÉCORESPONSABLES - "Entretien du cadre de vie et pratiques écoresponsablesEntretien du linge et pratiques écoresponsables " - 42 h"PERSONNE AGÉE EN SITUATION DE DÉPENDANCE : ACCOMPAGNEMENT PERSONNALISÉ " - "Les droits de la personne âgée dépendante et les fondements d'une démarche de bientraitanceComprendre les pathologies liées au vieillissement pour un accompagnement de qualité S'inscrire dans une démarche de projet personnalisé et travailler en collaboration pour mieux accompagner la personne en situation de dépendance - 56 h"PERSONNE EN SITUATION DE HANDICAP : PROJET ET ACCOMPAGNEMENT PERSONNALISÉ" - "Les droits de la personne en situation de handicap et les fondements d'une démarche de bientraitance Comprendre le handicap pour mieux accompagner la personne S'inscrire dans une démarche de projet personnalisé et travailler en collaboration pour mieux accompagner la personne en situation de dépendance - 56 hACTES DU QUOTIDIEN ET ACTIVITÉS DE L'ADULTE EN SITUATION DE DÉPENDANCE - "Accompagner une personne en situation de dépendance dans les actes d'hygiène et de confortTransferts et déplacements d'une personne en situation de dépendance Accompagner une personne en situation de dépendance dans ses loisirs" - 56 | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Assistant de vie dépendance et handicap</t>
+        </is>
+      </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10925810/true/false/false/true</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2369,32 +2361,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>INSUP AQUITAINE | 36 Chemin DE MACY | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2404,17 +2396,17 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | paysmontois@insup.org | nrousseau@insup.org</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2429,40 +2421,48 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0558068971</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr"/>
+          <t>0558068971</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T17" s="7" t="inlineStr"/>
+          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre équipe, Visite du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification visée, Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action. - 17 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Réaliser une prestation de nettoyage manuel - Environnement professionnel : le nettoyage industriel Prévention des risques : Règles d'hygiène et de sécurité, EPI, Gestuelle métier, Dysfonctionnements et risques associésNettoyage manuel : Techniques de nettoyage, Choix et utilisation des produits, Lavage des surfaces vitrées, Dépoussiérage des surfaces et sols, Nettoyage, Désinfection, Détartrage des sanitaires, Protocoles de bionettoyage en environnement spécifique Respect des standards de qualité : Contrôle de sa prestationIntégration des principes du développement durablePosture professionnelle adaptée - 245 hModule 4 CCP 2 Réaliser une prestation de nettoyage ou de remise en état mécanisée - Prévention des risques : Hygiène et Sécurité, Gestuelle, DysfonctionnementsRevêtements de sols : caractéristiquesProduits écologiques / écogestesUtilisation du matériel professionnel : Autolaveuse et monobrosseTechniques de nettoyage ou de remise en état mécanisé : Lavages mécanisés, méthode spray, lustrage et spray moquette - Remise en état - Récurage - Décapage - Métallisation - Shampoin | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
+        </is>
+      </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10925813/true/false/false/true</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2474,32 +2474,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40100 Dax</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>INSUP AQUITAINE | 3 Rue DES SALINES | 40100 Dax | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@greta-cfa-aquitaine.fr | paysdacquois@insup.org | landes@insup.org</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2534,12 +2534,12 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0558917868</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0558917868</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -2549,33 +2549,33 @@
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Module 1 Période d'intégration et bilans - Accueil : Identification des objectifs de formation, Rencontre équipe, Visite du centre, Positionnement : Evaluation des savoirs et compétences en lien avec les attendus de la certification visée, Bilan personnel et professionnelSynthèse du positionnement : Individualisation du parcours, Informations sur la VAE, Elaboration de l'annexe pédagogiqueFormalisation de l'engagement : Signature du contrat de formation et de l'annexe personnaliséeBilans intermédiaire et final : Point d'étape avec réajustement éventuel du parcours, Présentation du parcours à venir, Evaluation de l'action. - 17 hModule 2 Plateforme LMS - Présentation du LMS : prise en main, planning et organisationGestion de son profil Apprenant : mot de passe, adresse mail, etc.Prise de contact avec le tuteur de formation distantIdentification des outils Web 2.0 pouvant être utilisésParticipation aux forums, Wiki, bases documentaires, glossaires, partage de documents, évaluations par les pairs...Suivi des modules de formation en auto apprentissage accompagné, en individuel ou en activités de groupe (plénière et ateliers)Repérage de sa progression : jalons, badges numériques, compétences développées, savoirs acquis. - 4 hModule 3 CCP 1 Réaliser une prestation de nettoyage manuel - Environnement professionnel : le nettoyage industriel Prévention des risques : Règles d'hygiène et de sécurité, EPI, Gestuelle métier, Dysfonctionnements et risques associésNettoyage manuel : Techniques de nettoyage, Choix et utilisation des produits, Lavage des surfaces vitrées, Dépoussiérage des surfaces et sols, Nettoyage, Désinfection, Détartrage des sanitaires, Protocoles de bionettoyage en environnement spécifique Respect des standards de qualité : Contrôle de sa prestationIntégration des principes du développement durablePosture professionnelle adaptée - 245 hModule 4 CCP 2 Réaliser une prestation de nettoyage ou de remise en état mécanisée - Prévention des risques : Hygiène et Sécurité, Gestuelle, DysfonctionnementsRevêtements de sols : caractéristiquesProduits écologiques / écogestesUtilisation du matériel professionnel : Autolaveuse et monobrosseTechniques de nettoyage ou de remise en état mécanisé : Lavages mécanisés, méthode spray, lustrage et spray moquette - Remise en état - Récurage - Décapage - Métallisation - Shampoin | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10925829/true/false/false/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2587,32 +2587,32 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
+          <t>Agent(e) de maintenance des bâtiments (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2622,17 +2622,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2647,12 +2647,12 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -2662,33 +2662,33 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>TP AMB Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP AMB Bloc de compétences : Assurer la maintenance courante des aménagements intérieurs d'un bâtiment - Effectuer la maintenance améliorative courante des aménagements intérieurs d'un bâtiment Effectuer la maintenance améliorative courante des revêtements intérieurs d'un bâtiment Effectuer la maintenance préventive courante des menuiseries et fermetures d'un bâtiment Effectuer la maintenance corrective courante des aménagements intérieurs d'un bâtiment - 280 hTP AMB Période 1 en entreprise - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 70 hTP AMB Bloc de compétences : Assurer la maintenance courante de l'installation et des équipements électriques d'un bâtiment - Effectuer la maintenance améliorative courante d'une installation électrique monophasée d'un bâtiment Effectuer la maintenance préventive courante de l'installation et des équipements électriques d'un bâtiment Effectuer la maintenance corrective courante de l'installation et des équipements électriques d'un bâtiment - 175 hTP AMB Bloc de compétences : Assurer la maintenance courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment - Effectuer la maintenance améliorative courante de l'installation sanitaire d'un bâtiment Effectuer la maintenance préventive courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment Effectuer la maintenance corrective courante de l'installation et des équipements thermiques et sanitaires d'un bâtiment - 140 hTP AMB Période 2 en entreprise - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP AMB Période de certification - Epreuve de certification - 35 hTP AMB Sensibi | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de maintenance des bâtiments</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10928110/true/false/false/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2700,32 +2700,32 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Action Préparatoire aux métiers du BTP [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>AFEC</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2735,17 +2735,17 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>cergy@afec.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>cergy@afec.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2760,48 +2760,40 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0143388881</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0143388881</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0619257169</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Période d'intégration - Intégrer son groupe et sa formationS'approprier le cadre et les objectifs de la formation préparatoire Développer sa culture numérique et prendre en main la plateforme MètisDécouvrir la boîte à outils numériqueDécouvrir Mètis et se repérer dans son parcoursPasser les tests de positionnementPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une continuité de parcours certifiant ou une perspective d'emploi, un contrat en alternanceInitier son portefeuille de compétences - 35 hModule 1 : Découverte des métiers du secteur BTP et de leurs évolutions - Immersions sur les plateaux de formation - Découverte des métiers Les travaux publics : Canalisateur, maçon voirie réseaux divers, conducteur d'engins... Le gros oeuvre : Maçon, charpentier, couvreur zingueur... Le second oeuvre : Peintre, Carreleur, agent de maintenance des bâtiments, plombier, électricien, menuisier...Visites d'entreprises : Préparer, réaliser et exploiter une visite en entreprise Participation à des évènementiels Salons, jobs dating à partir d'une préparation collectiveMatinale entreprise (témoignages professionnels)BILAN INDIVIDUEL D'ORIENTATION - 70 hModule 2 : Acquérir le socle des connaissances nécessaires pour aller vers les métiers de l'industrie - Se remettre à niveau en mathématiquesUtiliser le système métriqueApprendre à lire des documents techniques, des plans....Développer sa communication écrite, son expression orale, comprendre les règles et instructionsTravailler en équipe et adopter la posture professionnelle attendueBILAN INDIVIDUEL D'ORIENTATION - 70 hModule 3 : Acquérir les bases des connaissances techniques et les gestes professionnels d'un métier - Réaliser un ouvrage simple en tenant compte des exigences de sécurité Identifier le matériel et les équipements nécessaires à la réalisation d'un ouvrage simplePréparer la matière nécessaire à la réalisation d'un ouvrage simpleRéaliser un ouvrage simpleMaintenir, l'organisation et la propreté du poste de travailTravailler en sécurité et conformément à la réglementation Repérer les risques liés à l'exercice des métiers de l'industrie Se sensibiliser au développement durable dans les métiers du BTPBILAN INDIVIDUEL D'ORIENTATION - 105 hModule 4 : Acco | Organisme | DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE | http://www.afpa.fr | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10928111/true/false/false/true</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -2813,32 +2805,32 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Monteur, monteuse en installation thermique et sanitaire (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>CROIX ROUGE FRANCAISE (Croix-Rouge Compétence (ex IRFSS) - Site de Lons-le-Saunier)</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>39000 Lons-le-Saunier</t>
+          <t>40000 Mont-de-Marsan</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>155 Chemin de Chaudon | https://competence.croix-rouge.fr/formations-bourgogne-franche-comte/ | 39000 Lons-le-Saunier | France</t>
+          <t>AFPA ACCES A L' EMPLOI | 245 Rue de la Caserne Bosquet | 40000 Mont-de-Marsan | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2848,17 +2840,17 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>https://competence.croix-rouge.fr/formations-bourgogne-franche-comte/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>lonslesaunier.competence-bfc@croix-rouge.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>lonslesaunier.competence-bfc@croix-rouge.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formation-mont_de_marsan@afpa.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2873,12 +2865,12 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0384472887</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0384472887</t>
+          <t>0619257169</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -2899,22 +2891,22 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travailLa formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) ; la formation clinique de 2 100 heures le travail personnel complémentaire est estimé à 900 heures environ, soit 300 heures par an | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>TP ITS Période d'intégration - Intégrer son groupe et sa formationS'inscrire dans une perspective d'emploiPréciser ses besoins de formation et contractualiser son parcours personnaliséDévelopper son autonomie en formationS'approprier les objectifs de la formation et repérer son futur environnement professionnel - 35 hTP ITS Bloc de compétences : Réaliser des installations sanitaire de bâtiments - Installer des équipements de renouvellement d'air dans des locaux d'habitation Effectuer l'analyse et établir le mode opératoireInstaller un système d'extraction dans des bâtiments à usage d'habitation individuelle et collectifsInstaller des appareils sanitaires Effectuer l' analyse de la mise en oeuvre de travaux d'installation d'appareil sanitaireInstaller des équipements de production d'eau chaude sanitaireRéaliser l'installation d'un équipement de production ECS solaire individuel et collectif, à gaz - 350 hTP ITS Période en entreprise-1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 70 hTP ITS Bloc de Compétences : Réaliser des installations de chauffage dans des locaux d'habitation - Installer des émetteurs de chaleur en tube cuivre et matériaux de synthèse Effectuer l' analyse de la mise en oeuvre de travaux de chauffageRéaliser l'installation d' un plancher chauffant basse température Modifier un réseau de chauffage existant Établir un mode opératoire pour intervenir sur une installation de chauffage existanteInstaller un générateur de chauffage dans des locaux d'habitation - 350 hTP ITS Période en entreprise-2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 105 hTP ITS Période de Certification - Certification - 35 hTP ITS Sensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'a | Validation | Type de validation : | Diplôme autres ministères | Certifications :</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certifications : | Titre professionnel plombier chauffagiste</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10825378/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10928127/true/false/false/true</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-40&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr">
@@ -2926,32 +2918,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>CROIX ROUGE FRANCAISE (Croix-Rouge Compétence (ex IRFSS) - Site de Lons-le-Saunier)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>39000 Lons-le-Saunier</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>155 Chemin de Chaudon | https://competence.croix-rouge.fr/formations-bourgogne-franche-comte/ | 39000 Lons-le-Saunier | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2961,17 +2953,17 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://competence.croix-rouge.fr/formations-bourgogne-franche-comte/</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>lonslesaunier.competence-bfc@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>lonslesaunier.competence-bfc@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2986,40 +2978,48 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0384472887</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr"/>
+          <t>0384472887</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr"/>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travailLa formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) ; la formation clinique de 2 100 heures le travail personnel complémentaire est estimé à 900 heures environ, soit 300 heures par an | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+        </is>
+      </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10825378/true/false/false/true</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-38&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-39&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-17
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-41&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-18
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-42&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-19
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-43&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-22
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-44&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-46&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-26
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-49&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-28
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-50&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-09-29
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-51&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-52&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>